<commit_message>
feat(precios): núcleo ENCE 100% ADIF + tabla precios base canónica + fixes menú
- ENCE: núcleo CAC# con precios BPA reales (CAC010/020/030/040/050/170) + SAI
  COA220 6h — sin estimaciones. 1 ENCE €824.643 = $899K USD / $3.955M COP;
  5 ENCE $4,49M USD / $19.775M COP. Actualizado HTML, Excel y generador.
- Precios_Base_ADIF_BPA_2026.md: tabla canónica validable (códigos paramétricos,
  €, COP, URLs, versión BPA v1.4.0). Catálogo CAC# (17) + SAI COA#. Correcciones.
  precios_Adif_COMPLETO.md §2 marcado SUPERSEDED.
- Menú: corregido ?v= duplicado preexistente en INDICE_Documentos_Servidos;
  navMap del sidebar con resaltado activo de Apartadero y ENCE.
- roadmap.md: sesión 2026-05-23 documentada.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/IX_WBS_Planificacion/Baseline_ENCE_ADIF.xlsx
+++ b/IX_WBS_Planificacion/Baseline_ENCE_ADIF.xlsx
@@ -73,7 +73,7 @@
       <sz val="8.5"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -88,11 +88,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0014304A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FBE9D0"/>
       </patternFill>
     </fill>
     <fill>
@@ -137,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -173,17 +168,15 @@
     <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -195,32 +188,22 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -594,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -670,7 +653,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>CAC020$</t>
+          <t>CAC020caa</t>
         </is>
       </c>
       <c r="D5" s="6" t="n">
@@ -696,53 +679,53 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Armario energía + bastidores + controlador de objetos + cableado red local</t>
+          <t>Armario de distribución de energía</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>CAC010/030/040/050$</t>
+          <t>CAC010ca</t>
         </is>
       </c>
       <c r="D6" s="10" t="n">
-        <v>150000</v>
+        <v>36806.72</v>
       </c>
       <c r="E6" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>150000</v>
+        <v>36807</v>
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>⚠ estimado</t>
+          <t>✅ ADIF</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Aparatos de vía</t>
+          <t>Núcleo enclavamiento</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Motor eléctrico de aguja (con cerrojo)</t>
+          <t>Bastidor de equipos de enclavamiento</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>CFA010$</t>
+          <t>CAC030caa</t>
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>10624.66</v>
+        <v>16399.36</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>84997</v>
+        <v>16399</v>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
@@ -751,31 +734,31 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>Aparatos de vía</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>Comprobador de aguja</t>
-        </is>
-      </c>
-      <c r="C8" s="13" t="inlineStr">
-        <is>
-          <t>CFA040$</t>
-        </is>
-      </c>
-      <c r="D8" s="14" t="n">
-        <v>4963.85</v>
-      </c>
-      <c r="E8" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="F8" s="16" t="n">
-        <v>39711</v>
-      </c>
-      <c r="G8" s="15" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Núcleo enclavamiento</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Cableado red local del enclavamiento</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>CAC040ca</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>5689.43</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="12" t="n">
+        <v>5689</v>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
         <is>
           <t>✅ ADIF</t>
         </is>
@@ -784,27 +767,27 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Señalización</t>
+          <t>Núcleo enclavamiento</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Señal alta LED 3 focos</t>
+          <t>Controlador de objetos 160E/128S</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>CCA040$</t>
+          <t>CAC050ca</t>
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>7934.23</v>
+        <v>33919.15</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>95211</v>
+        <v>33919</v>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
@@ -813,31 +796,31 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
-        <is>
-          <t>Detección de tren</t>
-        </is>
-      </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>Sensor de rueda contador de ejes</t>
-        </is>
-      </c>
-      <c r="C10" s="13" t="inlineStr">
-        <is>
-          <t>CBB030$</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="n">
-        <v>8286.120000000001</v>
-      </c>
-      <c r="E10" s="15" t="n">
-        <v>9</v>
-      </c>
-      <c r="F10" s="16" t="n">
-        <v>74575</v>
-      </c>
-      <c r="G10" s="15" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Núcleo enclavamiento</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Firewall de enclavamiento</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>CAC170</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>6885.21</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="12" t="n">
+        <v>6885</v>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
         <is>
           <t>✅ ADIF</t>
         </is>
@@ -846,27 +829,27 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Detección de tren</t>
+          <t>Aparatos de vía</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Evaluador 8 contadores de ejes</t>
+          <t>Motor eléctrico de aguja (con cerrojo)</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>CBB040$</t>
+          <t>CFA010$</t>
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>13398.59</v>
+        <v>10624.66</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>26797</v>
+        <v>84997</v>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
@@ -875,31 +858,31 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>Armarios y cajas</t>
-        </is>
-      </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>Armario de señalización (grande)</t>
-        </is>
-      </c>
-      <c r="C12" s="13" t="inlineStr">
-        <is>
-          <t>CDB010$</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="n">
-        <v>4151.33</v>
-      </c>
-      <c r="E12" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="F12" s="16" t="n">
-        <v>16605</v>
-      </c>
-      <c r="G12" s="15" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Aparatos de vía</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Comprobador de aguja</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>CFA040$</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>4963.85</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="F12" s="12" t="n">
+        <v>39711</v>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
         <is>
           <t>✅ ADIF</t>
         </is>
@@ -908,27 +891,27 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Armarios y cajas</t>
+          <t>Señalización</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Caja de terminales 50 bornas</t>
+          <t>Señal alta LED 3 focos</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>CDA010$</t>
+          <t>CCA040$</t>
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>1066.04</v>
+        <v>7934.23</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>10660</v>
+        <v>95211</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
@@ -937,31 +920,31 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>Caseta técnica prefabricada</t>
-        </is>
-      </c>
-      <c r="C14" s="13" t="inlineStr">
-        <is>
-          <t>TMI010</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="n">
-        <v>7180.94</v>
-      </c>
-      <c r="E14" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" s="16" t="n">
-        <v>7181</v>
-      </c>
-      <c r="G14" s="15" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Detección de tren</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Sensor de rueda contador de ejes</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>CBB030$</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>8286.120000000001</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="F14" s="12" t="n">
+        <v>74575</v>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
         <is>
           <t>✅ ADIF</t>
         </is>
@@ -970,27 +953,27 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Cableado</t>
+          <t>Detección de tren</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Cable de señalización 7x4x0.9 (m)</t>
+          <t>Evaluador 8 contadores de ejes</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>CEA030$</t>
+          <t>CBB040$</t>
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>11.67</v>
+        <v>13398.59</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>2000</v>
+        <v>2</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>23340</v>
+        <v>26797</v>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
@@ -999,31 +982,31 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
-        <is>
-          <t>Cableado</t>
-        </is>
-      </c>
-      <c r="B16" s="13" t="inlineStr">
-        <is>
-          <t>Cable F.O. 48 fibras canalización (m)</t>
-        </is>
-      </c>
-      <c r="C16" s="13" t="inlineStr">
-        <is>
-          <t>TCJ010$</t>
-        </is>
-      </c>
-      <c r="D16" s="14" t="n">
-        <v>5.48</v>
-      </c>
-      <c r="E16" s="15" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F16" s="16" t="n">
-        <v>5480</v>
-      </c>
-      <c r="G16" s="15" t="inlineStr">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Armarios y cajas</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Armario de señalización (grande)</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>CDB010$</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>4151.33</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F16" s="12" t="n">
+        <v>16605</v>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
         <is>
           <t>✅ ADIF</t>
         </is>
@@ -1032,130 +1015,254 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
+          <t>Armarios y cajas</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Caja de terminales 50 bornas</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>CDA010$</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>1066.04</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F17" s="8" t="n">
+        <v>10660</v>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>✅ ADIF</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Caseta técnica prefabricada</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>TMI010</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>7180.94</v>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="12" t="n">
+        <v>7181</v>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>✅ ADIF</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Cableado</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Cable de señalización 7x4x0.9 (m)</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>CEA030$</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>11.67</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>23340</v>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>✅ ADIF</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Cableado</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Cable F.O. 48 fibras canalización (m)</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>TCJ010$</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="n">
+        <v>5.48</v>
+      </c>
+      <c r="E20" s="11" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F20" s="12" t="n">
+        <v>5480</v>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>✅ ADIF</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
           <t>Energía</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>SAI 1 kVA (ENCE requiere mayor autonomía → COA200)</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>COA090$</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="n">
-        <v>2115.07</v>
-      </c>
-      <c r="E17" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F17" s="8" t="n">
-        <v>4230</v>
-      </c>
-      <c r="G17" s="7" t="inlineStr">
-        <is>
-          <t>✅ ADIF</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>SAI 20 kVA · 6h (autonomía DBCD ≥4h)</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>COA220ckea</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>32077.37</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>32077</v>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>✅ ADIF</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
         <is>
           <t>Subtotal EQUIPO (suministro + montaje)</t>
         </is>
       </c>
-      <c r="B18" s="18" t="n"/>
-      <c r="C18" s="18" t="n"/>
-      <c r="D18" s="18" t="n"/>
-      <c r="E18" s="18" t="n"/>
-      <c r="F18" s="19" t="n">
-        <v>656794</v>
-      </c>
-      <c r="G18" s="20" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="17" t="inlineStr">
+      <c r="B22" s="14" t="n"/>
+      <c r="C22" s="14" t="n"/>
+      <c r="D22" s="14" t="n"/>
+      <c r="E22" s="14" t="n"/>
+      <c r="F22" s="15" t="n">
+        <v>634341</v>
+      </c>
+      <c r="G22" s="16" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>Ingeniería + integración + pruebas + safety case (30%)</t>
         </is>
       </c>
-      <c r="B19" s="18" t="n"/>
-      <c r="C19" s="18" t="n"/>
-      <c r="D19" s="18" t="n"/>
-      <c r="E19" s="18" t="n"/>
-      <c r="F19" s="19" t="n">
-        <v>197038</v>
-      </c>
-      <c r="G19" s="20" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="21" t="inlineStr">
+      <c r="B23" s="14" t="n"/>
+      <c r="C23" s="14" t="n"/>
+      <c r="D23" s="14" t="n"/>
+      <c r="E23" s="14" t="n"/>
+      <c r="F23" s="15" t="n">
+        <v>190302</v>
+      </c>
+      <c r="G23" s="16" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>TOTAL ENCE tipo</t>
         </is>
       </c>
-      <c r="B20" s="22" t="n"/>
-      <c r="C20" s="22" t="n"/>
-      <c r="D20" s="22" t="n"/>
-      <c r="E20" s="22" t="n"/>
-      <c r="F20" s="23" t="n">
-        <v>853832</v>
-      </c>
-      <c r="G20" s="24" t="inlineStr">
-        <is>
-          <t>≈ $930,677 USD · $4,094 M COP</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="25" t="inlineStr">
+      <c r="B24" s="18" t="n"/>
+      <c r="C24" s="18" t="n"/>
+      <c r="D24" s="18" t="n"/>
+      <c r="E24" s="18" t="n"/>
+      <c r="F24" s="19" t="n">
+        <v>824643</v>
+      </c>
+      <c r="G24" s="20" t="inlineStr">
+        <is>
+          <t>≈ $898,861 USD · $3,954 M COP</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="inlineStr">
         <is>
           <t>Cantidades = ENCE PROMEDIO (referencia Ardanuy ÷ 5 estaciones): 8 desvíos motorizados, 12 señales, 9 contadores de ejes. Ajustar por estación (La Dorada–México &gt; Zapatosa).</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="25" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="21" t="inlineStr">
         <is>
           <t>Precios ADIF = suministro + montaje, costes indirectos 6% incluidos. Referencia europea; aplicar factores LFC (trocha 914, logística, MO).</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="25" t="inlineStr">
-        <is>
-          <t>PENDIENTE BPA: armario energía (CAC010$), bastidores (CAC030$), controlador de objetos (CAC050$) y cableado red local (CAC040$) — estimados en €150.000; consultar bpa.adif.es para cerrar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="25" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>Núcleo CAC 100% precios ADIF reales (sin estimaciones): UCP CAC020 + CAC010/030/040/050 + firewall CAC170. Catálogo completo CAC# (17 ítems) en Precios_Base_ADIF_BPA_2026.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="21" t="inlineStr">
         <is>
           <t>Detección por contador de ejes (Ardanuy). Alternativa: circuito de vía AF (CBC030$ €7.938/u) — solución mixta según TCO Detección.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="25" t="inlineStr">
-        <is>
-          <t>ENERGÍA: el ENCE exige autonomía 4 h+ (BCD §10.5) → usar SAI COA200$ (1 h) o banco mayor; COA090 (15 min) es solo referencia de orden.</t>
+    <row r="30">
+      <c r="A30" s="21" t="inlineStr">
+        <is>
+          <t>ENERGÍA: SAI COA220$ 6h/20 kVA (€32.077) cumple DBCD §10.5 (≥4h). COA200 (1h) y COA210 (2h) no alcanzan.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="A22:G22"/>
-    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A27:G27"/>
     <mergeCell ref="A26:G26"/>
-    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A30:G30"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A25:G25"/>
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="A23:G23"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A28:G28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1219,42 +1326,42 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="26" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>Bottom-up ADIF (este modelo)</t>
         </is>
       </c>
-      <c r="B5" s="27" t="n">
-        <v>930677</v>
-      </c>
-      <c r="C5" s="28" t="n">
-        <v>4095</v>
-      </c>
-      <c r="D5" s="28" t="n">
-        <v>20475</v>
-      </c>
-      <c r="E5" s="26" t="inlineStr">
-        <is>
-          <t>Suma de partidas BPA + 30% ingeniería. Núcleo CAC parcialmente estimado.</t>
+      <c r="B5" s="23" t="n">
+        <v>898861</v>
+      </c>
+      <c r="C5" s="24" t="n">
+        <v>3955</v>
+      </c>
+      <c r="D5" s="24" t="n">
+        <v>19775</v>
+      </c>
+      <c r="E5" s="22" t="inlineStr">
+        <is>
+          <t>Suma de partidas BPA reales + 30% ingeniería. Núcleo CAC 100% ADIF.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Ardanuy (consultor diseño)</t>
         </is>
       </c>
-      <c r="B6" s="29" t="n">
+      <c r="B6" s="25" t="n">
         <v>869377</v>
       </c>
-      <c r="C6" s="30" t="n">
+      <c r="C6" s="26" t="n">
         <v>3825</v>
       </c>
-      <c r="D6" s="30" t="n">
+      <c r="D6" s="26" t="n">
         <v>19126</v>
       </c>
-      <c r="E6" s="13" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>5 × $869.377 USD = $4,35M. Coincide con la Conceptual LFC.</t>
         </is>
@@ -1266,13 +1373,13 @@
           <t>WBS v3.0 (línea base antigua)</t>
         </is>
       </c>
-      <c r="B7" s="31" t="n">
+      <c r="B7" s="27" t="n">
         <v>181818</v>
       </c>
-      <c r="C7" s="32" t="n">
+      <c r="C7" s="28" t="n">
         <v>800</v>
       </c>
-      <c r="D7" s="32" t="n">
+      <c r="D7" s="28" t="n">
         <v>4000</v>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -1282,42 +1389,42 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>DT-COMS-2026-007 (LFC v2)</t>
         </is>
       </c>
-      <c r="B8" s="29" t="n">
+      <c r="B8" s="25" t="n">
         <v>454545</v>
       </c>
-      <c r="C8" s="30" t="n">
+      <c r="C8" s="26" t="n">
         <v>2000</v>
       </c>
-      <c r="D8" s="30" t="n">
+      <c r="D8" s="26" t="n">
         <v>10000</v>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>$2.000M COP/ENCE — entre el WBS viejo y el bottom-up real.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="inlineStr">
-        <is>
-          <t>LECTURA: el baseline bottom-up ADIF (~$930,677 USD/ENCE) CONFIRMA a Ardanuy ($869k) y expone que el WBS v3.0 ($800M COP) subestima el ENCE ~4–5×.</t>
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>LECTURA: el baseline bottom-up ADIF (~$898,861 USD/ENCE) CONFIRMA a Ardanuy ($869k) y expone que el WBS v3.0 ($800M COP) subestima el ENCE ~4–5×.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="25" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>Las cantidades por ENCE son promedio (Ardanuy ÷ 5). El desglose real por estación lo fija la ingeniería de detalle; La Dorada–México y Barrancabermeja serán mayores que Zapatosa.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="25" t="inlineStr">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>Para defensa ante Interventoría: cerrar los precios CAC010/030/040/050 en BPA y confirmar cantidades por estación (nº de desvíos, señales y contadores).</t>
         </is>

</xml_diff>

<commit_message>
fix(ence): núcleo CAC completo — añade registrador jurídico (CAC070) + interfaz CTC (CAC080)
Revisión del catálogo CAC# del BPA: el núcleo tipo omitía dos módulos vitales y
no-duplicativos. Añadidos con precio ADIF real:
- CAC070 Registrador jurídico €23.352,44 (obligatorio en sistemas vitales)
- CAC080 Control de interfaz a CTC serie €25.505,19 (enlace ENCE↔CCO)
Módulos de mando CAC130-160 excluidos (duplicarían controlador de objetos/campo);
CAC060/090/140 marcados como añadidos por estación.
Nuevo ENCE: €888.158 = $968K USD / $4.260M COP; 5 ENCE $4,84M USD / $21.298M COP.
Actualizado HTML, Excel, generador y Precios_Base_ADIF_BPA_2026.md.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/IX_WBS_Planificacion/Baseline_ENCE_ADIF.xlsx
+++ b/IX_WBS_Planificacion/Baseline_ENCE_ADIF.xlsx
@@ -577,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -803,22 +803,22 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Firewall de enclavamiento</t>
+          <t>Registrador jurídico</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>CAC170</t>
+          <t>CAC070</t>
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>6885.21</v>
+        <v>23352.44</v>
       </c>
       <c r="E10" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>6885</v>
+        <v>23352</v>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
@@ -829,27 +829,27 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Aparatos de vía</t>
+          <t>Núcleo enclavamiento</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Motor eléctrico de aguja (con cerrojo)</t>
+          <t>Control de interfaz a CTC (serie)</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>CFA010$</t>
+          <t>CAC080</t>
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>10624.66</v>
+        <v>25505.19</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>84997</v>
+        <v>25505</v>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
@@ -860,27 +860,27 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>Aparatos de vía</t>
+          <t>Núcleo enclavamiento</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Comprobador de aguja</t>
+          <t>Firewall de enclavamiento</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>CFA040$</t>
+          <t>CAC170</t>
         </is>
       </c>
       <c r="D12" s="10" t="n">
-        <v>4963.85</v>
+        <v>6885.21</v>
       </c>
       <c r="E12" s="11" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F12" s="12" t="n">
-        <v>39711</v>
+        <v>6885</v>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
@@ -891,27 +891,27 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Señalización</t>
+          <t>Aparatos de vía</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Señal alta LED 3 focos</t>
+          <t>Motor eléctrico de aguja (con cerrojo)</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>CCA040$</t>
+          <t>CFA010$</t>
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>7934.23</v>
+        <v>10624.66</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>95211</v>
+        <v>84997</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
@@ -922,27 +922,27 @@
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>Detección de tren</t>
+          <t>Aparatos de vía</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Sensor de rueda contador de ejes</t>
+          <t>Comprobador de aguja</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>CBB030$</t>
+          <t>CFA040$</t>
         </is>
       </c>
       <c r="D14" s="10" t="n">
-        <v>8286.120000000001</v>
+        <v>4963.85</v>
       </c>
       <c r="E14" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F14" s="12" t="n">
-        <v>74575</v>
+        <v>39711</v>
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
@@ -953,27 +953,27 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Detección de tren</t>
+          <t>Señalización</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Evaluador 8 contadores de ejes</t>
+          <t>Señal alta LED 3 focos</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>CBB040$</t>
+          <t>CCA040$</t>
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>13398.59</v>
+        <v>7934.23</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>26797</v>
+        <v>95211</v>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
@@ -984,27 +984,27 @@
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>Armarios y cajas</t>
+          <t>Detección de tren</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Armario de señalización (grande)</t>
+          <t>Sensor de rueda contador de ejes</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>CDB010$</t>
+          <t>CBB030$</t>
         </is>
       </c>
       <c r="D16" s="10" t="n">
-        <v>4151.33</v>
+        <v>8286.120000000001</v>
       </c>
       <c r="E16" s="11" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>16605</v>
+        <v>74575</v>
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
@@ -1015,27 +1015,27 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Armarios y cajas</t>
+          <t>Detección de tren</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Caja de terminales 50 bornas</t>
+          <t>Evaluador 8 contadores de ejes</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>CDA010$</t>
+          <t>CBB040$</t>
         </is>
       </c>
       <c r="D17" s="6" t="n">
-        <v>1066.04</v>
+        <v>13398.59</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>10660</v>
+        <v>26797</v>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
@@ -1046,27 +1046,27 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Armarios y cajas</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Caseta técnica prefabricada</t>
+          <t>Armario de señalización (grande)</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>TMI010</t>
+          <t>CDB010$</t>
         </is>
       </c>
       <c r="D18" s="10" t="n">
-        <v>7180.94</v>
+        <v>4151.33</v>
       </c>
       <c r="E18" s="11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>7181</v>
+        <v>16605</v>
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
@@ -1077,27 +1077,27 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Cableado</t>
+          <t>Armarios y cajas</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Cable de señalización 7x4x0.9 (m)</t>
+          <t>Caja de terminales 50 bornas</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>CEA030$</t>
+          <t>CDA010$</t>
         </is>
       </c>
       <c r="D19" s="6" t="n">
-        <v>11.67</v>
+        <v>1066.04</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>2000</v>
+        <v>10</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>23340</v>
+        <v>10660</v>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
@@ -1108,27 +1108,27 @@
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Cableado</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Cable F.O. 48 fibras canalización (m)</t>
+          <t>Caseta técnica prefabricada</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>TCJ010$</t>
+          <t>TMI010</t>
         </is>
       </c>
       <c r="D20" s="10" t="n">
-        <v>5.48</v>
+        <v>7180.94</v>
       </c>
       <c r="E20" s="11" t="n">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>5480</v>
+        <v>7181</v>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
@@ -1139,129 +1139,199 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
+          <t>Cableado</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Cable de señalización 7x4x0.9 (m)</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>CEA030$</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>11.67</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>23340</v>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>✅ ADIF</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Cableado</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Cable F.O. 48 fibras canalización (m)</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>TCJ010$</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="n">
+        <v>5.48</v>
+      </c>
+      <c r="E22" s="11" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F22" s="12" t="n">
+        <v>5480</v>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>✅ ADIF</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
           <t>Energía</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>SAI 20 kVA · 6h (autonomía DBCD ≥4h)</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>COA220ckea</t>
         </is>
       </c>
-      <c r="D21" s="6" t="n">
+      <c r="D23" s="6" t="n">
         <v>32077.37</v>
       </c>
-      <c r="E21" s="7" t="n">
+      <c r="E23" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="F21" s="8" t="n">
+      <c r="F23" s="8" t="n">
         <v>32077</v>
       </c>
-      <c r="G21" s="7" t="inlineStr">
-        <is>
-          <t>✅ ADIF</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="13" t="inlineStr">
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>✅ ADIF</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
         <is>
           <t>Subtotal EQUIPO (suministro + montaje)</t>
         </is>
       </c>
-      <c r="B22" s="14" t="n"/>
-      <c r="C22" s="14" t="n"/>
-      <c r="D22" s="14" t="n"/>
-      <c r="E22" s="14" t="n"/>
-      <c r="F22" s="15" t="n">
-        <v>634341</v>
-      </c>
-      <c r="G22" s="16" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="B24" s="14" t="n"/>
+      <c r="C24" s="14" t="n"/>
+      <c r="D24" s="14" t="n"/>
+      <c r="E24" s="14" t="n"/>
+      <c r="F24" s="15" t="n">
+        <v>683199</v>
+      </c>
+      <c r="G24" s="16" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
         <is>
           <t>Ingeniería + integración + pruebas + safety case (30%)</t>
         </is>
       </c>
-      <c r="B23" s="14" t="n"/>
-      <c r="C23" s="14" t="n"/>
-      <c r="D23" s="14" t="n"/>
-      <c r="E23" s="14" t="n"/>
-      <c r="F23" s="15" t="n">
-        <v>190302</v>
-      </c>
-      <c r="G23" s="16" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="17" t="inlineStr">
+      <c r="B25" s="14" t="n"/>
+      <c r="C25" s="14" t="n"/>
+      <c r="D25" s="14" t="n"/>
+      <c r="E25" s="14" t="n"/>
+      <c r="F25" s="15" t="n">
+        <v>204960</v>
+      </c>
+      <c r="G25" s="16" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>TOTAL ENCE tipo</t>
         </is>
       </c>
-      <c r="B24" s="18" t="n"/>
-      <c r="C24" s="18" t="n"/>
-      <c r="D24" s="18" t="n"/>
-      <c r="E24" s="18" t="n"/>
-      <c r="F24" s="19" t="n">
-        <v>824643</v>
-      </c>
-      <c r="G24" s="20" t="inlineStr">
-        <is>
-          <t>≈ $898,861 USD · $3,954 M COP</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="21" t="inlineStr">
-        <is>
-          <t>Cantidades = ENCE PROMEDIO (referencia Ardanuy ÷ 5 estaciones): 8 desvíos motorizados, 12 señales, 9 contadores de ejes. Ajustar por estación (La Dorada–México &gt; Zapatosa).</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="21" t="inlineStr">
-        <is>
-          <t>Precios ADIF = suministro + montaje, costes indirectos 6% incluidos. Referencia europea; aplicar factores LFC (trocha 914, logística, MO).</t>
+      <c r="B26" s="18" t="n"/>
+      <c r="C26" s="18" t="n"/>
+      <c r="D26" s="18" t="n"/>
+      <c r="E26" s="18" t="n"/>
+      <c r="F26" s="19" t="n">
+        <v>888158</v>
+      </c>
+      <c r="G26" s="20" t="inlineStr">
+        <is>
+          <t>≈ $968,092 USD · $4,259 M COP</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="21" t="inlineStr">
         <is>
-          <t>Núcleo CAC 100% precios ADIF reales (sin estimaciones): UCP CAC020 + CAC010/030/040/050 + firewall CAC170. Catálogo completo CAC# (17 ítems) en Precios_Base_ADIF_BPA_2026.md.</t>
+          <t>Cantidades = ENCE PROMEDIO (referencia Ardanuy ÷ 5 estaciones): 8 desvíos motorizados, 12 señales, 9 contadores de ejes. Ajustar por estación (La Dorada–México &gt; Zapatosa).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="21" t="inlineStr">
         <is>
-          <t>Detección por contador de ejes (Ardanuy). Alternativa: circuito de vía AF (CBC030$ €7.938/u) — solución mixta según TCO Detección.</t>
+          <t>Precios ADIF = suministro + montaje, costes indirectos 6% incluidos. Referencia europea; aplicar factores LFC (trocha 914, logística, MO).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="21" t="inlineStr">
         <is>
+          <t>Núcleo CAC 100% precios ADIF reales: UCP CAC020 + CAC010/030/040/050 + registrador CAC070 + interfaz CTC CAC080 + firewall CAC170. Catálogo completo (17 módulos) en Precios_Base_ADIF_BPA_2026.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="21" t="inlineStr">
+        <is>
+          <t>Módulos CAC por estación (no en el tipo): CAC060 interfaz a ENCE de otra tecnología (frontera FENOCO: García Cadena/Chiriguaná), CAC140 control de mando local (operación degradada), CAC090 rack adicional. Los módulos de mando CAC130-160 no se suman para no duplicar el controlador de objetos / equipo de campo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="21" t="inlineStr">
+        <is>
+          <t>Detección por contador de ejes (Ardanuy). Alternativa: circuito de vía AF (CBC030$ €7.938/u) — solución mixta según TCO Detección.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="21" t="inlineStr">
+        <is>
           <t>ENERGÍA: SAI COA220$ 6h/20 kVA (€32.077) cumple DBCD §10.5 (≥4h). COA200 (1h) y COA210 (2h) no alcanzan.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
+    <mergeCell ref="A32:G32"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A26:E26"/>
     <mergeCell ref="A24:E24"/>
-    <mergeCell ref="A27:G27"/>
-    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="A25:E25"/>
     <mergeCell ref="A30:G30"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A23:E23"/>
     <mergeCell ref="A29:G29"/>
-    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A33:G33"/>
     <mergeCell ref="A28:G28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1332,13 +1402,13 @@
         </is>
       </c>
       <c r="B5" s="23" t="n">
-        <v>898861</v>
+        <v>968092</v>
       </c>
       <c r="C5" s="24" t="n">
-        <v>3955</v>
+        <v>4260</v>
       </c>
       <c r="D5" s="24" t="n">
-        <v>19775</v>
+        <v>21298</v>
       </c>
       <c r="E5" s="22" t="inlineStr">
         <is>
@@ -1412,7 +1482,7 @@
     <row r="10">
       <c r="A10" s="21" t="inlineStr">
         <is>
-          <t>LECTURA: el baseline bottom-up ADIF (~$898,861 USD/ENCE) CONFIRMA a Ardanuy ($869k) y expone que el WBS v3.0 ($800M COP) subestima el ENCE ~4–5×.</t>
+          <t>LECTURA: el baseline bottom-up ADIF (~$968,092 USD/ENCE) CONFIRMA a Ardanuy ($869k) y expone que el WBS v3.0 ($800M COP) subestima el ENCE ~4–5×.</t>
         </is>
       </c>
     </row>

</xml_diff>